<commit_message>
feat(phase-4.1): Add UserID and Mobile columns to Excel test data
- Created ExcelDataUpdater utility to add UserID/Mobile columns programmatically
- Updated registration_testdata.xlsx HostYourBusiness sheet:
  - Added UserID column (position 1)
  - Added Mobile column (position 2)
  - Populated with sample data:
    * Row 1 (Architect): USER001 | 9876543210
    * Row 2 (Interior): USER001 | 9876543211
- Preserved all existing business data (shifted right by 2 columns)
- Columns now: UserID, Mobile, Profession, BusinessName, AboutBusiness, ...

Excel structure now ready for multi-user data-driven tests.
Both rows assigned to USER001 (tests multi-business in same session).

Closes Phase 4.1: Update Excel test data
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/registration_testdata.xlsx
+++ b/src/test/resources/testdata/registration_testdata.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\DialinArch-Playwright_Automation\playwright-java-framework-main\src\test\resources\testdata\"/>
     </mc:Choice>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="52">
   <si>
     <t>FirstName</t>
   </si>
@@ -163,13 +163,29 @@
   </si>
   <si>
     <t>Home Renovation</t>
+  </si>
+  <si>
+    <t>UserID</t>
+  </si>
+  <si>
+    <t>Mobile</t>
+  </si>
+  <si>
+    <t>USER001</t>
+  </si>
+  <si>
+    <t>9876543210</t>
+  </si>
+  <si>
+    <t>9876543211</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -194,6 +210,11 @@
       <b/>
       <sz val="12"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
     </font>
   </fonts>
   <fills count="4">
@@ -226,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -242,6 +263,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -559,10 +581,10 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="10.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="9.88671875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.6640625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="21.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -580,44 +602,44 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="2">
         <v>9876543212</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>7</v>
       </c>
       <c r="C3" s="3">
         <v>8765432112</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" t="s" s="0">
         <v>9</v>
       </c>
       <c r="C4" s="3">
         <v>7654321092</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" t="s" s="0">
         <v>12</v>
       </c>
     </row>
@@ -629,131 +651,152 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EC39A7C-5B22-4D23-910C-0F7195E8FFF4}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.109375" customWidth="1"/>
-    <col min="4" max="4" width="20.5546875" customWidth="1"/>
-    <col min="5" max="5" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.44140625" customWidth="1"/>
-    <col min="9" max="9" width="21.109375" customWidth="1"/>
-    <col min="10" max="10" width="27" customWidth="1"/>
-    <col min="11" max="11" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="8.13671875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="10.9296875"/>
+    <col min="3" max="3" customWidth="true" width="19.109375"/>
+    <col min="4" max="4" customWidth="true" width="20.5546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="16.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="12.0"/>
+    <col min="8" max="8" customWidth="true" width="20.44140625"/>
+    <col min="9" max="9" customWidth="true" width="21.109375"/>
+    <col min="10" max="10" customWidth="true" width="27.0"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="11.44140625"/>
+    <col min="12" max="12" customWidth="true" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" t="s" s="7">
+        <v>47</v>
+      </c>
+      <c r="B1" t="s" s="7">
+        <v>48</v>
+      </c>
+      <c r="C1" t="s" s="4">
         <v>13</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="D1" t="s" s="4">
         <v>16</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" t="s" s="4">
         <v>17</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="F1" t="s" s="4">
         <v>15</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" t="s" s="4">
         <v>14</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="H1" t="s" s="4">
         <v>18</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="I1" t="s" s="4">
         <v>19</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="J1" t="s" s="4">
         <v>20</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="K1" t="s" s="4">
         <v>21</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="L1" t="s" s="4">
         <v>22</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="M1" t="s" s="4">
         <v>30</v>
       </c>
-      <c r="L1" s="4"/>
+      <c r="N1" s="4"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C2" t="s" s="5">
         <v>23</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="D2" t="s" s="5">
         <v>29</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="E2" t="s" s="5">
         <v>24</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F2" t="s" s="5">
         <v>25</v>
       </c>
-      <c r="E2" s="5">
-        <v>411057</v>
-      </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" t="n" s="5">
+        <v>411057.0</v>
+      </c>
+      <c r="H2" t="s" s="5">
         <v>26</v>
       </c>
-      <c r="G2" s="5">
-        <v>10</v>
-      </c>
-      <c r="H2" s="5">
-        <v>500</v>
-      </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" t="n" s="5">
+        <v>10.0</v>
+      </c>
+      <c r="J2" t="n" s="5">
+        <v>500.0</v>
+      </c>
+      <c r="K2" t="s" s="5">
         <v>27</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="L2" t="s" s="5">
         <v>28</v>
       </c>
-      <c r="K2">
-        <v>10</v>
+      <c r="M2" t="n" s="0">
+        <v>10.0</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="C3" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="D3" t="s" s="5">
         <v>39</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s" s="0">
         <v>40</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s" s="0">
         <v>41</v>
       </c>
-      <c r="E3">
-        <v>411014</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="G3" t="n" s="0">
+        <v>411014.0</v>
+      </c>
+      <c r="H3" t="s" s="0">
         <v>42</v>
       </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
-      <c r="H3">
-        <v>6</v>
-      </c>
-      <c r="I3" t="s">
+      <c r="I3" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="J3" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="K3" t="s" s="0">
         <v>45</v>
       </c>
-      <c r="J3" t="s">
+      <c r="L3" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="K3">
-        <v>6</v>
+      <c r="M3" t="n" s="0">
+        <v>6.0</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="F13" t="s">
+      <c r="F13" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="H13" t="s" s="0">
         <v>44</v>
       </c>
     </row>
@@ -768,9 +811,9 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="27.88671875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="17.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
@@ -785,24 +828,24 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>35</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>36</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>37</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" t="s" s="0">
         <v>38</v>
       </c>
     </row>

</xml_diff>